<commit_message>
Corrige peso de referencia del HSS 10x10x5/16 y del PIPX7
HSS 10x10x5/16 pesa 40.35 lb/ft (60.0 kg/m), no 37.69. PIPX7 es tubo
3/4 in XS (2.19 kg/m).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014KBVAj2qFmD27bb5fprGRc
</commit_message>
<xml_diff>
--- a/Peso_Estructura_NOSE_DOCK_H5_H6_R2.4.xlsx
+++ b/Peso_Estructura_NOSE_DOCK_H5_H6_R2.4.xlsx
@@ -1028,11 +1028,11 @@
       </c>
       <c r="C5" s="23" t="n"/>
       <c r="D5" s="24" t="n">
-        <v>56.1</v>
+        <v>60</v>
       </c>
       <c r="E5" s="25" t="inlineStr">
         <is>
-          <t>AISC: 37.69 lb/ft (≈ 56.1 kg/m). Verifica con tu proveedor.</t>
+          <t>AISC: 40.35 lb/ft (≈ 60.0 kg/m), peso nominal. Verifica con tu proveedor.</t>
         </is>
       </c>
       <c r="F5" s="6">
@@ -1172,14 +1172,16 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Tubo PIPX7 (contraflambeos de techo)</t>
+          <t>Tubo 3/4" céd. 80 XS — PIPX7 (contraflambeos de techo)</t>
         </is>
       </c>
       <c r="C10" s="23" t="n"/>
-      <c r="D10" s="24" t="n"/>
+      <c r="D10" s="24" t="n">
+        <v>2.19</v>
+      </c>
       <c r="E10" s="25" t="inlineStr">
         <is>
-          <t>Revisa qué tubo es en tu catálogo STAAD / proveedor.</t>
+          <t>ASTM A53 3/4" XS: 1.47 lb/ft (≈ 2.19 kg/m).</t>
         </is>
       </c>
       <c r="F10" s="6">

</xml_diff>